<commit_message>
Actualización comensales y restaurante
</commit_message>
<xml_diff>
--- a/resources/Comensales - Tabla de Datos.xlsx
+++ b/resources/Comensales - Tabla de Datos.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BOOM\Documents\Programación 1\Corte 2\L26.2.p.c2.xx.comensales\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BOOM\Documents\Programación 1\Corte 2\L26.2.p.c2.18.comensales\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AC018B79-6536-4304-86BB-1BA7945B5F5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{082A9846-02CA-428F-B749-F6317B498998}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{6CBE7975-ED01-4762-9FF8-9CF4CEBDB024}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="64">
   <si>
     <t>COMENSALES</t>
   </si>
@@ -48,15 +48,9 @@
     <t>turnoComida</t>
   </si>
   <si>
-    <t>costo</t>
-  </si>
-  <si>
     <t>get edad()</t>
   </si>
   <si>
-    <t>costoFinal()</t>
-  </si>
-  <si>
     <t>aplicaDescuento()</t>
   </si>
   <si>
@@ -220,6 +214,9 @@
   </si>
   <si>
     <t>Porcentaje sin Descuento:</t>
+  </si>
+  <si>
+    <t>get costo()</t>
   </si>
 </sst>
 </file>
@@ -314,7 +311,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -352,9 +349,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -674,34 +668,33 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A56F2D2-B0C5-4D76-BA0B-4DE5F77CA7F2}">
-  <dimension ref="A1:O23"/>
+  <dimension ref="A1:N23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" customWidth="1"/>
     <col min="2" max="2" width="9.28515625" customWidth="1"/>
     <col min="3" max="3" width="8" customWidth="1"/>
-    <col min="4" max="4" width="7.140625" customWidth="1"/>
+    <col min="4" max="4" width="5.42578125" customWidth="1"/>
     <col min="5" max="5" width="16" customWidth="1"/>
     <col min="6" max="6" width="12.28515625" customWidth="1"/>
-    <col min="7" max="7" width="6.7109375" customWidth="1"/>
+    <col min="7" max="7" width="9.7109375" customWidth="1"/>
     <col min="8" max="8" width="10" customWidth="1"/>
-    <col min="9" max="9" width="11.42578125" customWidth="1"/>
-    <col min="10" max="10" width="17" customWidth="1"/>
-    <col min="11" max="11" width="14.28515625" customWidth="1"/>
-    <col min="12" max="12" width="14" customWidth="1"/>
-    <col min="13" max="13" width="11.7109375" customWidth="1"/>
-    <col min="14" max="14" width="15.28515625" customWidth="1"/>
+    <col min="9" max="9" width="17.140625" customWidth="1"/>
+    <col min="10" max="11" width="14.28515625" customWidth="1"/>
+    <col min="12" max="12" width="11.85546875" customWidth="1"/>
+    <col min="13" max="13" width="15.42578125" customWidth="1"/>
+    <col min="14" max="14" width="18" customWidth="1"/>
     <col min="15" max="15" width="17.7109375" customWidth="1"/>
     <col min="16" max="16" width="11.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="D1" s="1"/>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
@@ -724,42 +717,39 @@
         <v>7</v>
       </c>
       <c r="H3" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="I3" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="I3" s="2" t="s">
+      <c r="J3" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="K3" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="J3" s="2" t="s">
+      <c r="L3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="K3" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="L3" s="2" t="s">
+      <c r="M3" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M3" s="2" t="s">
+      <c r="N3" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="N3" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="O3" s="2" t="s">
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>16</v>
-      </c>
       <c r="B4" s="3" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C4" s="6">
         <v>111</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="E4" s="9">
         <v>18730</v>
@@ -767,46 +757,43 @@
       <c r="F4" s="6">
         <v>1</v>
       </c>
-      <c r="G4" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="H4" s="6">
+      <c r="G4" s="6">
         <v>75</v>
       </c>
-      <c r="I4" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="J4" s="6" t="b">
+      <c r="H4" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="I4" s="6" t="b">
         <v>1</v>
       </c>
+      <c r="J4" s="13">
+        <v>1</v>
+      </c>
       <c r="K4" s="13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L4" s="13">
         <v>0</v>
       </c>
       <c r="M4" s="13">
+        <v>1</v>
+      </c>
+      <c r="N4" s="13">
         <v>0</v>
       </c>
-      <c r="N4" s="13">
-        <v>1</v>
-      </c>
-      <c r="O4" s="13">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C5" s="7">
         <v>222</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="E5" s="11">
         <v>35875</v>
@@ -814,23 +801,23 @@
       <c r="F5" s="7">
         <v>3</v>
       </c>
-      <c r="G5" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="H5" s="7">
+      <c r="G5" s="7">
         <v>28</v>
       </c>
-      <c r="I5" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="J5" s="7" t="b">
+      <c r="H5" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="I5" s="7" t="b">
         <v>0</v>
       </c>
+      <c r="J5" s="14">
+        <v>0.5</v>
+      </c>
       <c r="K5" s="14">
+        <v>0</v>
+      </c>
+      <c r="L5" s="14">
         <v>0.5</v>
-      </c>
-      <c r="L5" s="14">
-        <v>0</v>
       </c>
       <c r="M5" s="14">
         <v>0.5</v>
@@ -838,22 +825,19 @@
       <c r="N5" s="14">
         <v>0.5</v>
       </c>
-      <c r="O5" s="14">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C6" s="6">
         <v>333</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="E6" s="9">
         <v>37576</v>
@@ -861,46 +845,43 @@
       <c r="F6" s="6">
         <v>2</v>
       </c>
-      <c r="G6" s="6" t="s">
+      <c r="G6" s="6">
+        <v>23</v>
+      </c>
+      <c r="H6" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="I6" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="J6" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="H6" s="6">
-        <v>23</v>
-      </c>
-      <c r="I6" s="6" t="s">
+      <c r="K6" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="J6" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="K6" s="6" t="s">
-        <v>42</v>
-      </c>
       <c r="L6" s="6" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="M6" s="6" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="N6" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="O6" s="6" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C7" s="7">
         <v>444</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="E7" s="11">
         <v>38943</v>
@@ -908,46 +889,43 @@
       <c r="F7" s="7">
         <v>2</v>
       </c>
-      <c r="G7" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="H7" s="7">
+      <c r="G7" s="7">
         <v>19</v>
       </c>
-      <c r="I7" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="J7" s="7" t="b">
+      <c r="H7" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="I7" s="7" t="b">
         <v>0</v>
       </c>
+      <c r="J7" s="14">
+        <v>0.25</v>
+      </c>
       <c r="K7" s="14">
+        <v>0.5</v>
+      </c>
+      <c r="L7" s="14">
         <v>0.25</v>
-      </c>
-      <c r="L7" s="14">
-        <v>0.5</v>
       </c>
       <c r="M7" s="14">
         <v>0.25</v>
       </c>
       <c r="N7" s="14">
-        <v>0.25</v>
-      </c>
-      <c r="O7" s="14">
         <v>0.75</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C8" s="6">
         <v>555</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="E8" s="9">
         <v>38355</v>
@@ -955,46 +933,43 @@
       <c r="F8" s="6">
         <v>1</v>
       </c>
-      <c r="G8" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="H8" s="6">
+      <c r="G8" s="6">
         <v>21</v>
       </c>
-      <c r="I8" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="J8" s="6" t="b">
+      <c r="H8" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="I8" s="6" t="b">
         <v>0</v>
+      </c>
+      <c r="J8" s="13">
+        <v>0.4</v>
       </c>
       <c r="K8" s="13">
         <v>0.4</v>
       </c>
       <c r="L8" s="13">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="M8" s="13">
         <v>0.2</v>
       </c>
       <c r="N8" s="13">
-        <v>0.2</v>
-      </c>
-      <c r="O8" s="13">
         <v>0.8</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C9" s="7">
         <v>666</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="E9" s="11">
         <v>15230</v>
@@ -1002,46 +977,43 @@
       <c r="F9" s="7">
         <v>1</v>
       </c>
-      <c r="G9" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="H9" s="7">
+      <c r="G9" s="7">
         <v>84</v>
       </c>
-      <c r="I9" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="J9" s="7" t="b">
+      <c r="H9" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="I9" s="7" t="b">
         <v>1</v>
       </c>
-      <c r="K9" s="14">
+      <c r="J9" s="14">
         <v>0.5</v>
       </c>
+      <c r="K9" s="7" t="s">
+        <v>40</v>
+      </c>
       <c r="L9" s="7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="M9" s="7" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="N9" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="O9" s="7" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C10" s="6">
         <v>777</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="E10" s="9">
         <v>30735</v>
@@ -1049,46 +1021,43 @@
       <c r="F10" s="6">
         <v>1</v>
       </c>
-      <c r="G10" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="H10" s="6">
+      <c r="G10" s="6">
         <v>42</v>
       </c>
-      <c r="I10" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="J10" s="6" t="b">
+      <c r="H10" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="I10" s="6" t="b">
         <v>0</v>
       </c>
+      <c r="J10" s="6" t="s">
+        <v>44</v>
+      </c>
       <c r="K10" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="L10" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="L10" s="6" t="s">
-        <v>47</v>
-      </c>
       <c r="M10" s="6" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="N10" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="O10" s="6" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C11" s="7">
         <v>888</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="E11" s="11">
         <v>37798</v>
@@ -1096,20 +1065,20 @@
       <c r="F11" s="7">
         <v>3</v>
       </c>
-      <c r="G11" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="H11" s="7">
+      <c r="G11" s="7">
         <v>22</v>
       </c>
-      <c r="I11" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="J11" s="7" t="b">
+      <c r="H11" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="I11" s="7" t="b">
         <v>0</v>
       </c>
+      <c r="J11" s="14">
+        <v>0.5</v>
+      </c>
       <c r="K11" s="14">
-        <v>0.5</v>
+        <v>0.25</v>
       </c>
       <c r="L11" s="14">
         <v>0.25</v>
@@ -1118,24 +1087,21 @@
         <v>0.25</v>
       </c>
       <c r="N11" s="14">
-        <v>0.25</v>
-      </c>
-      <c r="O11" s="14">
         <v>0.75</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C12" s="6">
         <v>999</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="E12" s="9">
         <v>24721</v>
@@ -1143,46 +1109,43 @@
       <c r="F12" s="6">
         <v>2</v>
       </c>
-      <c r="G12" s="6" t="s">
+      <c r="G12" s="6">
+        <v>58</v>
+      </c>
+      <c r="H12" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="I12" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="J12" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="K12" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="H12" s="6">
-        <v>58</v>
-      </c>
-      <c r="I12" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="J12" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="K12" s="6" t="s">
-        <v>43</v>
-      </c>
       <c r="L12" s="6" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="M12" s="6" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="N12" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="O12" s="6" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C13" s="8">
         <v>1000</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="E13" s="12">
         <v>34436</v>
@@ -1190,103 +1153,100 @@
       <c r="F13" s="10">
         <v>2</v>
       </c>
-      <c r="G13" s="10" t="s">
-        <v>40</v>
-      </c>
-      <c r="H13" s="10">
+      <c r="G13" s="10">
         <v>32</v>
       </c>
-      <c r="I13" s="8" t="s">
-        <v>40</v>
-      </c>
-      <c r="J13" s="10" t="b">
+      <c r="H13" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="I13" s="10" t="b">
         <v>0</v>
+      </c>
+      <c r="J13" s="15">
+        <v>0.4</v>
       </c>
       <c r="K13" s="15">
         <v>0.4</v>
       </c>
       <c r="L13" s="15">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="M13" s="15">
         <v>0.2</v>
       </c>
       <c r="N13" s="15">
-        <v>0.2</v>
-      </c>
-      <c r="O13" s="15">
         <v>0.8</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="E15" t="s">
+        <v>50</v>
+      </c>
+      <c r="I15" s="16" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="E16" t="s">
         <v>52</v>
       </c>
-      <c r="I15" s="16" t="s">
+      <c r="I16" s="16" t="s">
         <v>53</v>
-      </c>
-    </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="E16" t="s">
-        <v>54</v>
-      </c>
-      <c r="I16" s="17" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="17" spans="5:9" x14ac:dyDescent="0.25">
       <c r="E17" t="s">
-        <v>56</v>
-      </c>
-      <c r="I17" s="17" t="s">
-        <v>59</v>
+        <v>54</v>
+      </c>
+      <c r="I17" s="16" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="18" spans="5:9" x14ac:dyDescent="0.25">
       <c r="E18" t="s">
-        <v>57</v>
-      </c>
-      <c r="I18" s="17" t="s">
-        <v>58</v>
+        <v>55</v>
+      </c>
+      <c r="I18" s="16" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="19" spans="5:9" x14ac:dyDescent="0.25">
       <c r="E19" t="s">
-        <v>60</v>
-      </c>
-      <c r="I19" s="18">
+        <v>58</v>
+      </c>
+      <c r="I19" s="17">
         <v>0.4</v>
       </c>
     </row>
     <row r="20" spans="5:9" x14ac:dyDescent="0.25">
       <c r="E20" t="s">
-        <v>61</v>
-      </c>
-      <c r="I20" s="18">
+        <v>59</v>
+      </c>
+      <c r="I20" s="17">
         <v>0.4</v>
       </c>
     </row>
     <row r="21" spans="5:9" x14ac:dyDescent="0.25">
       <c r="E21" t="s">
-        <v>62</v>
-      </c>
-      <c r="I21" s="18">
+        <v>60</v>
+      </c>
+      <c r="I21" s="17">
         <v>0.2</v>
       </c>
     </row>
     <row r="22" spans="5:9" x14ac:dyDescent="0.25">
       <c r="E22" t="s">
-        <v>63</v>
-      </c>
-      <c r="I22" s="18">
+        <v>61</v>
+      </c>
+      <c r="I22" s="17">
         <v>0.2</v>
       </c>
     </row>
     <row r="23" spans="5:9" x14ac:dyDescent="0.25">
       <c r="E23" t="s">
-        <v>64</v>
-      </c>
-      <c r="I23" s="18">
+        <v>62</v>
+      </c>
+      <c r="I23" s="17">
         <v>0.8</v>
       </c>
     </row>

</xml_diff>